<commit_message>
Replace initial tool with updated ML prediction tool
</commit_message>
<xml_diff>
--- a/Paper_Final_Slim/Results.xlsx
+++ b/Paper_Final_Slim/Results.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table0_Dataset" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table2_PerformanceGrid" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table3_Calibration" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table5_PredictionInterval" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table5_UncertaintyBand" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table6_FeatureImportance" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table7_ResidualDiagnostics" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table8_Model_Mapping" sheetId="8" state="visible" r:id="rId8"/>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -484,6 +484,16 @@
           <t>Average_RMSE</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Average_MAE</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Average_Abs_MBE</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -492,29 +502,41 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.6588433009908246</v>
+        <v>0.7177140494134013</v>
       </c>
       <c r="C2" t="n">
-        <v>0.6395615228151718</v>
+        <v>0.6355021737473133</v>
       </c>
       <c r="D2" t="n">
-        <v>1.778517906770204</v>
+        <v>2.294659941613896</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1.236916447529437</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.1983209169621401</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>Extra Trees</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.6605001543167822</v>
+        <v>0.6821355550897124</v>
       </c>
       <c r="C3" t="n">
-        <v>0.6349853885395722</v>
+        <v>0.6252028524243306</v>
       </c>
       <c r="D3" t="n">
-        <v>1.731461221582002</v>
+        <v>2.303038046878246</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.214017291424684</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.2499008701157673</v>
       </c>
     </row>
     <row r="4">
@@ -524,13 +546,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.6726548508018902</v>
+        <v>0.7003086315947226</v>
       </c>
       <c r="C4" t="n">
-        <v>0.6332961555443842</v>
+        <v>0.588755930344165</v>
       </c>
       <c r="D4" t="n">
-        <v>1.669650378843211</v>
+        <v>2.381635960005238</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1.316249242853935</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.2612572986206682</v>
       </c>
     </row>
     <row r="5">
@@ -540,29 +568,41 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.6534109568028947</v>
+        <v>0.6665544853940772</v>
       </c>
       <c r="C5" t="n">
-        <v>0.6122227001219857</v>
+        <v>0.5879578572175619</v>
       </c>
       <c r="D5" t="n">
-        <v>1.720332648568558</v>
+        <v>2.385243086826437</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.320204775173636</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.3048796775303833</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Extra Trees</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.6622936990595961</v>
+        <v>0.6814004787404824</v>
       </c>
       <c r="C6" t="n">
-        <v>0.6032957542740199</v>
+        <v>0.5903135733010271</v>
       </c>
       <c r="D6" t="n">
-        <v>1.733707189384379</v>
+        <v>2.413956138620375</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.410018708614838</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.2413662630958594</v>
       </c>
     </row>
     <row r="7">
@@ -572,45 +612,63 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.6071658608528778</v>
+        <v>0.6371985880541122</v>
       </c>
       <c r="C7" t="n">
-        <v>0.5225877084101618</v>
+        <v>0.5344456612608836</v>
       </c>
       <c r="D7" t="n">
-        <v>2.104786026711884</v>
+        <v>2.748093038404734</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1.638247039463359</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.4341221036734692</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SVR</t>
+          <t>Decision Tree</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.4468964830601505</v>
+        <v>0.5280715259771757</v>
       </c>
       <c r="C8" t="n">
-        <v>0.4751758383420223</v>
+        <v>0.4557715254764485</v>
       </c>
       <c r="D8" t="n">
-        <v>2.720487488997076</v>
+        <v>2.980254803667611</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1.643981673474813</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.3416910342866544</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Decision Tree</t>
+          <t>Lasso</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.4948376623682623</v>
+        <v>0.5601900433231802</v>
       </c>
       <c r="C9" t="n">
-        <v>0.4749175731207354</v>
+        <v>0.4733367522497925</v>
       </c>
       <c r="D9" t="n">
-        <v>1.979842566399429</v>
+        <v>3.017550468662523</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1.950760754024824</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.4597872657121953</v>
       </c>
     </row>
     <row r="10">
@@ -620,45 +678,63 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.4852325662663484</v>
+        <v>0.5565248964329719</v>
       </c>
       <c r="C10" t="n">
-        <v>0.4745507290012085</v>
+        <v>0.4760057285878095</v>
       </c>
       <c r="D10" t="n">
-        <v>2.407569669426493</v>
+        <v>3.020017636152504</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1.946659795279215</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.4610699719692612</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Lasso</t>
+          <t>Linear Regression</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.4818427777526751</v>
+        <v>0.5538036306839876</v>
       </c>
       <c r="C11" t="n">
-        <v>0.4682976206533588</v>
+        <v>0.4725376463442398</v>
       </c>
       <c r="D11" t="n">
-        <v>2.391565246021147</v>
+        <v>3.023622621511223</v>
+      </c>
+      <c r="E11" t="n">
+        <v>2.015054614964733</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.4073936775234405</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Linear Regression</t>
+          <t>SVR</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.4897344864057274</v>
+        <v>0.5315777319969435</v>
       </c>
       <c r="C12" t="n">
-        <v>0.440561705494494</v>
+        <v>0.4837634341778113</v>
       </c>
       <c r="D12" t="n">
-        <v>2.40902256444171</v>
+        <v>3.073648260457993</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1.559455805330805</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.5848083512142283</v>
       </c>
     </row>
   </sheetData>
@@ -672,7 +748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -714,16 +790,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>206</v>
+        <v>236</v>
       </c>
       <c r="C2" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="D2" t="n">
-        <v>174</v>
+        <v>199</v>
       </c>
       <c r="E2" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="F2" t="n">
         <v>15</v>
@@ -732,20 +808,20 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GAMMA_WET</t>
+          <t>SP_GR</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>332</v>
+        <v>395</v>
       </c>
       <c r="C3" t="n">
-        <v>84</v>
+        <v>98</v>
       </c>
       <c r="D3" t="n">
-        <v>171</v>
+        <v>200</v>
       </c>
       <c r="E3" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="F3" t="n">
         <v>15</v>
@@ -754,20 +830,20 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GAMMA_DRY</t>
+          <t>COHESION</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>333</v>
+        <v>199</v>
       </c>
       <c r="C4" t="n">
-        <v>84</v>
+        <v>50</v>
       </c>
       <c r="D4" t="n">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="E4" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="F4" t="n">
         <v>15</v>
@@ -776,66 +852,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SP_GR</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>331</v>
+        <v>400</v>
       </c>
       <c r="C5" t="n">
-        <v>85</v>
+        <v>99</v>
       </c>
       <c r="D5" t="n">
-        <v>169</v>
+        <v>201</v>
       </c>
       <c r="E5" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="F5" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>COHESION</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>167</v>
-      </c>
-      <c r="C6" t="n">
-        <v>44</v>
-      </c>
-      <c r="D6" t="n">
-        <v>152</v>
-      </c>
-      <c r="E6" t="n">
-        <v>39</v>
-      </c>
-      <c r="F6" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>MC</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>334</v>
-      </c>
-      <c r="C7" t="n">
-        <v>85</v>
-      </c>
-      <c r="D7" t="n">
-        <v>172</v>
-      </c>
-      <c r="E7" t="n">
-        <v>43</v>
-      </c>
-      <c r="F7" t="n">
         <v>15</v>
       </c>
     </row>
@@ -850,7 +882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S14"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -863,15 +895,19 @@
       <c r="C1" s="1" t="n"/>
       <c r="D1" s="1" t="n"/>
       <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>MBE</t>
+        </is>
+      </c>
       <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>R2_test</t>
         </is>
       </c>
-      <c r="I1" s="1" t="n"/>
-      <c r="J1" s="1" t="n"/>
       <c r="K1" s="1" t="n"/>
       <c r="L1" s="1" t="n"/>
       <c r="M1" s="1" t="n"/>
@@ -883,8 +919,6 @@
       <c r="O1" s="1" t="n"/>
       <c r="P1" s="1" t="n"/>
       <c r="Q1" s="1" t="n"/>
-      <c r="R1" s="1" t="n"/>
-      <c r="S1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -894,92 +928,82 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>cohesion</t>
+          <t>Angle of Friction,ϕ</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>gamma_dry</t>
+          <t>Cohesion(KN/m2)</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>gamma_wet</t>
+          <t>Moisture Content(%)</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>mc</t>
+          <t>Specific Gravity</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>phi</t>
+          <t>Angle of Friction,ϕ</t>
         </is>
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
-          <t>sp_gr</t>
+          <t>Cohesion(KN/m2)</t>
         </is>
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t>cohesion</t>
+          <t>Moisture Content(%)</t>
         </is>
       </c>
       <c r="I2" s="1" t="inlineStr">
         <is>
-          <t>gamma_dry</t>
+          <t>Specific Gravity</t>
         </is>
       </c>
       <c r="J2" s="1" t="inlineStr">
         <is>
-          <t>gamma_wet</t>
+          <t>Angle of Friction,ϕ</t>
         </is>
       </c>
       <c r="K2" s="1" t="inlineStr">
         <is>
-          <t>mc</t>
+          <t>Cohesion(KN/m2)</t>
         </is>
       </c>
       <c r="L2" s="1" t="inlineStr">
         <is>
-          <t>phi</t>
+          <t>Moisture Content(%)</t>
         </is>
       </c>
       <c r="M2" s="1" t="inlineStr">
         <is>
-          <t>sp_gr</t>
+          <t>Specific Gravity</t>
         </is>
       </c>
       <c r="N2" s="1" t="inlineStr">
         <is>
-          <t>cohesion</t>
+          <t>Angle of Friction,ϕ</t>
         </is>
       </c>
       <c r="O2" s="1" t="inlineStr">
         <is>
-          <t>gamma_dry</t>
+          <t>Cohesion(KN/m2)</t>
         </is>
       </c>
       <c r="P2" s="1" t="inlineStr">
         <is>
-          <t>gamma_wet</t>
+          <t>Moisture Content(%)</t>
         </is>
       </c>
       <c r="Q2" s="1" t="inlineStr">
         <is>
-          <t>mc</t>
-        </is>
-      </c>
-      <c r="R2" s="1" t="inlineStr">
-        <is>
-          <t>phi</t>
-        </is>
-      </c>
-      <c r="S2" s="1" t="inlineStr">
-        <is>
-          <t>sp_gr</t>
+          <t>Specific Gravity</t>
         </is>
       </c>
     </row>
@@ -997,58 +1021,52 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.9118692776265316</v>
+        <v>1.395953185201958</v>
       </c>
       <c r="C4" t="n">
-        <v>0.7112124877325172</v>
+        <v>1.562908548263576</v>
       </c>
       <c r="D4" t="n">
-        <v>1.07495699622475</v>
+        <v>1.928963951284981</v>
       </c>
       <c r="E4" t="n">
-        <v>1.757143800348205</v>
+        <v>0.0598401053672323</v>
       </c>
       <c r="F4" t="n">
-        <v>1.956616425822371</v>
+        <v>-0.0486514814020102</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0681289538633912</v>
+        <v>-0.2627743178907392</v>
       </c>
       <c r="H4" t="n">
-        <v>0.9029273157386504</v>
+        <v>0.4682781490620471</v>
       </c>
       <c r="I4" t="n">
-        <v>0.5408736867361787</v>
+        <v>-0.013579719493764</v>
       </c>
       <c r="J4" t="n">
-        <v>0.5938666975497289</v>
+        <v>0.8341516662414941</v>
       </c>
       <c r="K4" t="n">
-        <v>0.6792368146880583</v>
+        <v>0.8302382722466113</v>
       </c>
       <c r="L4" t="n">
-        <v>0.80566275726729</v>
+        <v>0.5892259895641516</v>
       </c>
       <c r="M4" t="n">
-        <v>0.4304925339650411</v>
+        <v>0.6172402696013486</v>
       </c>
       <c r="N4" t="n">
-        <v>2.253417960786371</v>
+        <v>1.848213112605958</v>
       </c>
       <c r="O4" t="n">
-        <v>1.037216280797539</v>
+        <v>4.253334713116897</v>
       </c>
       <c r="P4" t="n">
-        <v>1.589872896327982</v>
+        <v>2.992115033452611</v>
       </c>
       <c r="Q4" t="n">
-        <v>2.722379189983279</v>
-      </c>
-      <c r="R4" t="n">
-        <v>2.953739524979518</v>
-      </c>
-      <c r="S4" t="n">
-        <v>0.1144815877465326</v>
+        <v>0.08497690728011539</v>
       </c>
     </row>
     <row r="5">
@@ -1058,58 +1076,52 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.6398416666666665</v>
+        <v>2.360029239766082</v>
       </c>
       <c r="C5" t="n">
-        <v>0.9206309523809518</v>
+        <v>2.065216666666667</v>
       </c>
       <c r="D5" t="n">
-        <v>1.368958333333333</v>
+        <v>2.073282828282829</v>
       </c>
       <c r="E5" t="n">
-        <v>2.036409803921568</v>
+        <v>0.0773979591836735</v>
       </c>
       <c r="F5" t="n">
-        <v>2.69076923076923</v>
+        <v>0.1907309941520464</v>
       </c>
       <c r="G5" t="n">
-        <v>0.08890000000000001</v>
+        <v>-0.5087766666666667</v>
       </c>
       <c r="H5" t="n">
-        <v>0.963255229355173</v>
+        <v>0.6625319865319862</v>
       </c>
       <c r="I5" t="n">
-        <v>0.2887189241635343</v>
+        <v>-0.0047244897959183</v>
       </c>
       <c r="J5" t="n">
-        <v>0.2246445006849166</v>
+        <v>0.5466392591017418</v>
       </c>
       <c r="K5" t="n">
-        <v>0.548711599979671</v>
+        <v>0.7068467723173959</v>
       </c>
       <c r="L5" t="n">
-        <v>0.704301619717515</v>
+        <v>0.5411071222171729</v>
       </c>
       <c r="M5" t="n">
-        <v>0.2393941003087637</v>
+        <v>0.3176929502723919</v>
       </c>
       <c r="N5" t="n">
-        <v>1.386407830145913</v>
+        <v>3.055754398102123</v>
       </c>
       <c r="O5" t="n">
-        <v>1.290992919521237</v>
+        <v>5.589294682148088</v>
       </c>
       <c r="P5" t="n">
-        <v>2.196739403512498</v>
+        <v>3.162514065924722</v>
       </c>
       <c r="Q5" t="n">
-        <v>3.22911448529629</v>
-      </c>
-      <c r="R5" t="n">
-        <v>3.643498952296353</v>
-      </c>
-      <c r="S5" t="n">
-        <v>0.1323018076242861</v>
+        <v>0.1134560684955108</v>
       </c>
     </row>
     <row r="6">
@@ -1119,58 +1131,52 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.750967344696971</v>
+        <v>1.351163673071574</v>
       </c>
       <c r="C6" t="n">
-        <v>0.6890427202801549</v>
+        <v>1.459367269841274</v>
       </c>
       <c r="D6" t="n">
-        <v>1.072163213741731</v>
+        <v>1.979279515707819</v>
       </c>
       <c r="E6" t="n">
-        <v>1.869970828268688</v>
+        <v>0.0662587070780687</v>
       </c>
       <c r="F6" t="n">
-        <v>2.023950408565794</v>
+        <v>-0.20168767752715</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0672291214069155</v>
+        <v>-0.3228806920634977</v>
       </c>
       <c r="H6" t="n">
-        <v>0.9354972923055964</v>
+        <v>0.4595023259409904</v>
       </c>
       <c r="I6" t="n">
-        <v>0.5710617545223295</v>
+        <v>-0.0155327849314312</v>
       </c>
       <c r="J6" t="n">
-        <v>0.5734270821495617</v>
+        <v>0.8351135596092467</v>
       </c>
       <c r="K6" t="n">
-        <v>0.6122195146733275</v>
+        <v>0.8394182829412534</v>
       </c>
       <c r="L6" t="n">
-        <v>0.8217759073923493</v>
+        <v>0.5487817131840259</v>
       </c>
       <c r="M6" t="n">
-        <v>0.4597806433144126</v>
+        <v>0.5052286646243231</v>
       </c>
       <c r="N6" t="n">
-        <v>1.836886003465461</v>
+        <v>1.842845650926761</v>
       </c>
       <c r="O6" t="n">
-        <v>1.00253748247224</v>
+        <v>4.13673514420411</v>
       </c>
       <c r="P6" t="n">
-        <v>1.629388865448128</v>
+        <v>3.135957391653286</v>
       </c>
       <c r="Q6" t="n">
-        <v>2.993293705925016</v>
-      </c>
-      <c r="R6" t="n">
-        <v>2.828638070924901</v>
-      </c>
-      <c r="S6" t="n">
-        <v>0.111499008070528</v>
+        <v>0.096614000728827</v>
       </c>
     </row>
     <row r="7">
@@ -1180,58 +1186,52 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.7590327921615819</v>
+        <v>1.483780962750824</v>
       </c>
       <c r="C7" t="n">
-        <v>0.7079753582861565</v>
+        <v>1.732679484650114</v>
       </c>
       <c r="D7" t="n">
-        <v>1.048090898407417</v>
+        <v>1.986403332861871</v>
       </c>
       <c r="E7" t="n">
-        <v>1.570144856623554</v>
+        <v>0.0621331911529307</v>
       </c>
       <c r="F7" t="n">
-        <v>1.939511494866129</v>
+        <v>-0.0574353299101051</v>
       </c>
       <c r="G7" t="n">
-        <v>0.07112620163172551</v>
+        <v>-0.4155995485693594</v>
       </c>
       <c r="H7" t="n">
-        <v>0.9201336659387306</v>
+        <v>0.5576384061818903</v>
       </c>
       <c r="I7" t="n">
-        <v>0.5473089473868399</v>
+        <v>-0.0143559098213179</v>
       </c>
       <c r="J7" t="n">
-        <v>0.6320157761366114</v>
+        <v>0.8269970662745736</v>
       </c>
       <c r="K7" t="n">
-        <v>0.6950104371596451</v>
+        <v>0.8116911167376286</v>
       </c>
       <c r="L7" t="n">
-        <v>0.8425789843870475</v>
+        <v>0.5670356467921436</v>
       </c>
       <c r="M7" t="n">
-        <v>0.3988812938024672</v>
+        <v>0.5955106965745444</v>
       </c>
       <c r="N7" t="n">
-        <v>2.043972776836965</v>
+        <v>1.887657616461183</v>
       </c>
       <c r="O7" t="n">
-        <v>1.029921652752768</v>
+        <v>4.479660188472549</v>
       </c>
       <c r="P7" t="n">
-        <v>1.513361580654458</v>
+        <v>3.071870320308673</v>
       </c>
       <c r="Q7" t="n">
-        <v>2.654598509919343</v>
-      </c>
-      <c r="R7" t="n">
-        <v>2.658431847909126</v>
-      </c>
-      <c r="S7" t="n">
-        <v>0.1176159049866038</v>
+        <v>0.08735571477854751</v>
       </c>
     </row>
     <row r="8">
@@ -1241,58 +1241,52 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1.883684588628254</v>
+        <v>2.047797018232086</v>
       </c>
       <c r="C8" t="n">
-        <v>0.8292716389842448</v>
+        <v>2.92880230335009</v>
       </c>
       <c r="D8" t="n">
-        <v>1.309241741927385</v>
+        <v>2.76195104366959</v>
       </c>
       <c r="E8" t="n">
-        <v>2.675444681797253</v>
+        <v>0.0644926508475288</v>
       </c>
       <c r="F8" t="n">
-        <v>2.158571119940561</v>
+        <v>-0.679029600683257</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0769571647539915</v>
+        <v>-0.7056432755586117</v>
       </c>
       <c r="H8" t="n">
-        <v>0.6935572728169761</v>
+        <v>0.4338078819198057</v>
       </c>
       <c r="I8" t="n">
-        <v>0.3667057071829361</v>
+        <v>-0.0206683046871068</v>
       </c>
       <c r="J8" t="n">
-        <v>0.3910889191854659</v>
+        <v>0.5892330356901492</v>
       </c>
       <c r="K8" t="n">
-        <v>0.3049513202522961</v>
+        <v>0.7288712193859772</v>
       </c>
       <c r="L8" t="n">
-        <v>0.7927523975129903</v>
+        <v>0.3738941867573009</v>
       </c>
       <c r="M8" t="n">
-        <v>0.3420010495653862</v>
+        <v>0.5487617314592936</v>
       </c>
       <c r="N8" t="n">
-        <v>4.00375866331586</v>
+        <v>2.908668616401567</v>
       </c>
       <c r="O8" t="n">
-        <v>1.218164728256613</v>
+        <v>5.375235269050122</v>
       </c>
       <c r="P8" t="n">
-        <v>1.94672695835929</v>
+        <v>3.694032186791496</v>
       </c>
       <c r="Q8" t="n">
-        <v>4.007411765567724</v>
-      </c>
-      <c r="R8" t="n">
-        <v>3.050274567818337</v>
-      </c>
-      <c r="S8" t="n">
-        <v>0.1230547928090541</v>
+        <v>0.0922658024069084</v>
       </c>
     </row>
     <row r="9">
@@ -1302,58 +1296,52 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2.133092732095085</v>
+        <v>1.770436142801671</v>
       </c>
       <c r="C9" t="n">
-        <v>0.7656522871177073</v>
+        <v>2.654826137483665</v>
       </c>
       <c r="D9" t="n">
-        <v>1.161998898689003</v>
+        <v>2.061830691192172</v>
       </c>
       <c r="E9" t="n">
-        <v>1.969842907380435</v>
+        <v>0.06589518637592739</v>
       </c>
       <c r="F9" t="n">
-        <v>2.137241487283829</v>
+        <v>-0.2131533454953326</v>
       </c>
       <c r="G9" t="n">
-        <v>0.0740201011723849</v>
+        <v>-0.9032891519136176</v>
       </c>
       <c r="H9" t="n">
-        <v>0.7390892956292676</v>
+        <v>0.6134797771012011</v>
       </c>
       <c r="I9" t="n">
-        <v>0.5514282324861532</v>
+        <v>-0.0065661401837256</v>
       </c>
       <c r="J9" t="n">
-        <v>0.59776674469462</v>
+        <v>0.7129863758925647</v>
       </c>
       <c r="K9" t="n">
-        <v>0.5907166800080919</v>
+        <v>0.7283692490911209</v>
       </c>
       <c r="L9" t="n">
-        <v>0.7814220629299422</v>
+        <v>0.5624307156058723</v>
       </c>
       <c r="M9" t="n">
-        <v>0.3825721493691919</v>
+        <v>0.5450080116268907</v>
       </c>
       <c r="N9" t="n">
-        <v>3.694359722028762</v>
+        <v>2.431351487897789</v>
       </c>
       <c r="O9" t="n">
-        <v>1.025225032000557</v>
+        <v>5.380208847859516</v>
       </c>
       <c r="P9" t="n">
-        <v>1.582220806528859</v>
+        <v>3.088163044082966</v>
       </c>
       <c r="Q9" t="n">
-        <v>3.075164697689387</v>
-      </c>
-      <c r="R9" t="n">
-        <v>3.132545137506191</v>
-      </c>
-      <c r="S9" t="n">
-        <v>0.1192007645175451</v>
+        <v>0.0926487737786638</v>
       </c>
     </row>
     <row r="10">
@@ -1363,58 +1351,52 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1.935524927895637</v>
+        <v>2.113772690226595</v>
       </c>
       <c r="C10" t="n">
-        <v>0.8064219410472087</v>
+        <v>3.074618148374864</v>
       </c>
       <c r="D10" t="n">
-        <v>1.29451851553937</v>
+        <v>2.80309585708195</v>
       </c>
       <c r="E10" t="n">
-        <v>2.69077247352685</v>
+        <v>0.06873176417552281</v>
       </c>
       <c r="F10" t="n">
-        <v>2.092321710389855</v>
+        <v>-0.5581225791328052</v>
       </c>
       <c r="G10" t="n">
-        <v>0.0711558050068047</v>
+        <v>-0.6317287721044603</v>
       </c>
       <c r="H10" t="n">
-        <v>0.6966370444617369</v>
+        <v>0.4216432508531769</v>
       </c>
       <c r="I10" t="n">
-        <v>0.362966881442234</v>
+        <v>-0.0180801080033195</v>
       </c>
       <c r="J10" t="n">
-        <v>0.3749251894652237</v>
+        <v>0.5901189962424195</v>
       </c>
       <c r="K10" t="n">
-        <v>0.279999568300076</v>
+        <v>0.7280498854483342</v>
       </c>
       <c r="L10" t="n">
-        <v>0.7881814399822339</v>
+        <v>0.3680175259675502</v>
       </c>
       <c r="M10" t="n">
-        <v>0.4356967947828597</v>
+        <v>0.5290281150776466</v>
       </c>
       <c r="N10" t="n">
-        <v>3.983588825715401</v>
+        <v>2.905530149938844</v>
       </c>
       <c r="O10" t="n">
-        <v>1.221755320555</v>
+        <v>5.38337074749953</v>
       </c>
       <c r="P10" t="n">
-        <v>1.972395955660102</v>
+        <v>3.711327883360409</v>
       </c>
       <c r="Q10" t="n">
-        <v>4.078709138665588</v>
-      </c>
-      <c r="R10" t="n">
-        <v>3.083728835376308</v>
-      </c>
-      <c r="S10" t="n">
-        <v>0.1139573106778624</v>
+        <v>0.0942617052461127</v>
       </c>
     </row>
     <row r="11">
@@ -1424,58 +1406,52 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.761748684376112</v>
+        <v>1.435253689780009</v>
       </c>
       <c r="C11" t="n">
-        <v>0.7250046794042395</v>
+        <v>1.668526422222223</v>
       </c>
       <c r="D11" t="n">
-        <v>1.117207413548754</v>
+        <v>2.109716561648228</v>
       </c>
       <c r="E11" t="n">
-        <v>1.812802683965487</v>
+        <v>0.06732242704408389</v>
       </c>
       <c r="F11" t="n">
-        <v>2.037051282051279</v>
+        <v>-0.2478691172375384</v>
       </c>
       <c r="G11" t="n">
-        <v>0.06922814940253311</v>
+        <v>-0.493362155555552</v>
       </c>
       <c r="H11" t="n">
-        <v>0.9391177335718704</v>
+        <v>0.4613589650473251</v>
       </c>
       <c r="I11" t="n">
-        <v>0.5294777269934378</v>
+        <v>-0.0169284722811177</v>
       </c>
       <c r="J11" t="n">
-        <v>0.5726486034491109</v>
+        <v>0.8096487785636283</v>
       </c>
       <c r="K11" t="n">
-        <v>0.6520454348870466</v>
+        <v>0.8231665125897154</v>
       </c>
       <c r="L11" t="n">
-        <v>0.8120120922783911</v>
+        <v>0.5531069860041868</v>
       </c>
       <c r="M11" t="n">
-        <v>0.4151641496375116</v>
+        <v>0.4802956644187786</v>
       </c>
       <c r="N11" t="n">
-        <v>1.78459075043385</v>
+        <v>1.980041645789636</v>
       </c>
       <c r="O11" t="n">
-        <v>1.050009737193451</v>
+        <v>4.341021364116558</v>
       </c>
       <c r="P11" t="n">
-        <v>1.630874972846936</v>
+        <v>3.120890922247739</v>
       </c>
       <c r="Q11" t="n">
-        <v>2.835421492102382</v>
-      </c>
-      <c r="R11" t="n">
-        <v>2.905086935457196</v>
-      </c>
-      <c r="S11" t="n">
-        <v>0.1160120033775352</v>
+        <v>0.0990184151518138</v>
       </c>
     </row>
     <row r="12">
@@ -1485,58 +1461,52 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1.909347724587846</v>
+        <v>2.047726079428202</v>
       </c>
       <c r="C12" t="n">
-        <v>0.8087352445101836</v>
+        <v>2.902096110135199</v>
       </c>
       <c r="D12" t="n">
-        <v>1.286337553733387</v>
+        <v>2.768795116601125</v>
       </c>
       <c r="E12" t="n">
-        <v>2.670224238457061</v>
+        <v>0.06802187495233369</v>
       </c>
       <c r="F12" t="n">
-        <v>2.180395678878518</v>
+        <v>-0.676272982226342</v>
       </c>
       <c r="G12" t="n">
-        <v>0.0729481348201458</v>
+        <v>-0.7131791449694228</v>
       </c>
       <c r="H12" t="n">
-        <v>0.6823904494656523</v>
+        <v>0.4363133368136028</v>
       </c>
       <c r="I12" t="n">
-        <v>0.3750916547020665</v>
+        <v>-0.0185144238676773</v>
       </c>
       <c r="J12" t="n">
-        <v>0.3953301618592361</v>
+        <v>0.5903705418017298</v>
       </c>
       <c r="K12" t="n">
-        <v>0.3039394212162869</v>
+        <v>0.7282400298159646</v>
       </c>
       <c r="L12" t="n">
-        <v>0.787547192150693</v>
+        <v>0.3717486622729768</v>
       </c>
       <c r="M12" t="n">
-        <v>0.3670965182041551</v>
+        <v>0.5357403518412163</v>
       </c>
       <c r="N12" t="n">
-        <v>4.076054748089747</v>
+        <v>2.904638445554755</v>
       </c>
       <c r="O12" t="n">
-        <v>1.210072511791685</v>
+        <v>5.381488423206038</v>
       </c>
       <c r="P12" t="n">
-        <v>1.939935351749181</v>
+        <v>3.700356084524394</v>
       </c>
       <c r="Q12" t="n">
-        <v>4.010327835602065</v>
-      </c>
-      <c r="R12" t="n">
-        <v>3.088342185633636</v>
-      </c>
-      <c r="S12" t="n">
-        <v>0.1206853836926469</v>
+        <v>0.0935875913248297</v>
       </c>
     </row>
     <row r="13">
@@ -1546,58 +1516,52 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1.524856290482301</v>
+        <v>1.654311100579277</v>
       </c>
       <c r="C13" t="n">
-        <v>0.7368596238282701</v>
+        <v>2.364229852448529</v>
       </c>
       <c r="D13" t="n">
-        <v>1.189640395646184</v>
+        <v>2.132950111605769</v>
       </c>
       <c r="E13" t="n">
-        <v>2.333788520370175</v>
+        <v>0.0863321566896441</v>
       </c>
       <c r="F13" t="n">
-        <v>2.197407860924456</v>
+        <v>0.0333253114080366</v>
       </c>
       <c r="G13" t="n">
-        <v>0.07789978794421321</v>
+        <v>-1.39452579949821</v>
       </c>
       <c r="H13" t="n">
-        <v>0.4786064045766988</v>
+        <v>0.9022941346333661</v>
       </c>
       <c r="I13" t="n">
-        <v>0.4181447535721201</v>
+        <v>-0.0090881593173002</v>
       </c>
       <c r="J13" t="n">
-        <v>0.4339798977595666</v>
+        <v>0.7319496521118936</v>
       </c>
       <c r="K13" t="n">
-        <v>0.33920446003348</v>
+        <v>0.6185094182398896</v>
       </c>
       <c r="L13" t="n">
-        <v>0.6385355602213609</v>
+        <v>0.452000988580473</v>
       </c>
       <c r="M13" t="n">
-        <v>0.3729078221976768</v>
+        <v>0.3238508690555178</v>
       </c>
       <c r="N13" t="n">
-        <v>5.222471494125363</v>
+        <v>2.349658132337963</v>
       </c>
       <c r="O13" t="n">
-        <v>1.167644695235222</v>
+        <v>6.376047995242817</v>
       </c>
       <c r="P13" t="n">
-        <v>1.876912523570656</v>
+        <v>3.455943984796793</v>
       </c>
       <c r="Q13" t="n">
-        <v>3.907418326414601</v>
-      </c>
-      <c r="R13" t="n">
-        <v>4.028347853762098</v>
-      </c>
-      <c r="S13" t="n">
-        <v>0.1201300408745172</v>
+        <v>0.1129429294544014</v>
       </c>
     </row>
     <row r="14">
@@ -1607,65 +1571,60 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.5976784110069275</v>
+        <v>1.711451921964947</v>
       </c>
       <c r="C14" t="n">
-        <v>0.6707290999094645</v>
+        <v>1.806323441505432</v>
       </c>
       <c r="D14" t="n">
-        <v>1.061856111798968</v>
+        <v>2.059045430193043</v>
       </c>
       <c r="E14" t="n">
-        <v>1.956498992022346</v>
+        <v>0.0632540407959296</v>
       </c>
       <c r="F14" t="n">
-        <v>2.003699717154869</v>
+        <v>-0.0035200018631784</v>
       </c>
       <c r="G14" t="n">
-        <v>0.06970833138858561</v>
+        <v>-0.376269136238098</v>
       </c>
       <c r="H14" t="n">
-        <v>0.9522802496977084</v>
+        <v>0.5717494540744363</v>
       </c>
       <c r="I14" t="n">
-        <v>0.5864556334907429</v>
+        <v>-0.013926460207725</v>
       </c>
       <c r="J14" t="n">
-        <v>0.6448601969505057</v>
+        <v>0.7690719454712212</v>
       </c>
       <c r="K14" t="n">
-        <v>0.5806736900644364</v>
+        <v>0.8304832975642269</v>
       </c>
       <c r="L14" t="n">
-        <v>0.78470486474343</v>
+        <v>0.548958743698621</v>
       </c>
       <c r="M14" t="n">
-        <v>0.41402629095387</v>
+        <v>0.5770879282278605</v>
       </c>
       <c r="N14" t="n">
-        <v>1.579946253171683</v>
+        <v>2.180895413895649</v>
       </c>
       <c r="O14" t="n">
-        <v>0.9843834145113878</v>
+        <v>4.25026408279954</v>
       </c>
       <c r="P14" t="n">
-        <v>1.486715191516062</v>
+        <v>3.135342152166724</v>
       </c>
       <c r="Q14" t="n">
-        <v>3.112665225007869</v>
-      </c>
-      <c r="R14" t="n">
-        <v>3.108932440067201</v>
-      </c>
-      <c r="S14" t="n">
-        <v>0.1161248052178091</v>
+        <v>0.0893229056195874</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="N1:S1"/>
-    <mergeCell ref="H1:M1"/>
-    <mergeCell ref="B1:G1"/>
+  <mergeCells count="4">
+    <mergeCell ref="J1:M1"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="N1:Q1"/>
+    <mergeCell ref="F1:I1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1677,7 +1636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1725,158 +1684,104 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Gradient Boosting</t>
+          <t>Extra Trees</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.798</v>
+        <v>0.8639</v>
       </c>
       <c r="D2" t="n">
-        <v>7.01</v>
+        <v>4.6649</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9199000000000001</v>
+        <v>0.9154</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.1926</v>
+        <v>-0.2017</v>
       </c>
       <c r="G2" t="n">
-        <v>0.202</v>
+        <v>0.1361</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GAMMA_WET</t>
+          <t>SP_GR</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.7071</v>
+        <v>0.5798</v>
       </c>
       <c r="D3" t="n">
-        <v>6.1752</v>
+        <v>1.126</v>
       </c>
       <c r="E3" t="n">
-        <v>0.8062</v>
+        <v>0.7945</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0146</v>
+        <v>-0.0136</v>
       </c>
       <c r="G3" t="n">
-        <v>0.2929</v>
+        <v>0.4202</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GAMMA_DRY</t>
+          <t>COHESION</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>Extra Trees</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.5934</v>
+        <v>0.7871</v>
       </c>
       <c r="D4" t="n">
-        <v>6.4409</v>
+        <v>1.0284</v>
       </c>
       <c r="E4" t="n">
-        <v>0.7667</v>
+        <v>0.9188</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0555</v>
+        <v>-0.3229</v>
       </c>
       <c r="G4" t="n">
-        <v>0.4066</v>
+        <v>0.2129</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SP_GR</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Extra Trees</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.5286</v>
+        <v>0.589</v>
       </c>
       <c r="D5" t="n">
-        <v>1.2769</v>
+        <v>13.9367</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6885</v>
+        <v>0.7743</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0135</v>
+        <v>0.4683</v>
       </c>
       <c r="G5" t="n">
-        <v>0.4714</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>COHESION</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Decision Tree</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>0.9323</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0.1235</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0.9825</v>
-      </c>
-      <c r="F6" t="n">
-        <v>-0.2182</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0.0677</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>MC</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Gradient Boosting</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>0.724</v>
-      </c>
-      <c r="D7" t="n">
-        <v>9.171200000000001</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0.8345</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0.0917</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.276</v>
+        <v>0.411</v>
       </c>
     </row>
   </sheetData>
@@ -1890,7 +1795,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1921,7 +1826,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Mean_PI_Width</t>
+          <t>Mean_Uncertainty_Band_Width</t>
         </is>
       </c>
     </row>
@@ -1933,152 +1838,100 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Gradient Boosting</t>
+          <t>Extra Trees</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Residual Bootstrap</t>
+          <t>Residual Bootstrap Uncertainty Band (in-sample, not an independent PI)</t>
         </is>
       </c>
       <c r="D2" t="n">
         <v>95</v>
       </c>
       <c r="E2" t="n">
-        <v>96.15000000000001</v>
+        <v>94.73999999999999</v>
       </c>
       <c r="F2" t="n">
-        <v>12.976</v>
+        <v>8.3757</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GAMMA_WET</t>
+          <t>SP_GR</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Residual Bootstrap</t>
+          <t>Residual Bootstrap Uncertainty Band (in-sample, not an independent PI)</t>
         </is>
       </c>
       <c r="D3" t="n">
         <v>95</v>
       </c>
       <c r="E3" t="n">
-        <v>95.23999999999999</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>6.0478</v>
+        <v>0.3268</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GAMMA_DRY</t>
+          <t>COHESION</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>Extra Trees</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Residual Bootstrap</t>
+          <t>Residual Bootstrap Uncertainty Band (in-sample, not an independent PI)</t>
         </is>
       </c>
       <c r="D4" t="n">
         <v>95</v>
       </c>
       <c r="E4" t="n">
-        <v>94.05</v>
+        <v>96</v>
       </c>
       <c r="F4" t="n">
-        <v>4.1396</v>
+        <v>14.8146</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SP_GR</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Extra Trees</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Residual Bootstrap</t>
+          <t>Residual Bootstrap Uncertainty Band (in-sample, not an independent PI)</t>
         </is>
       </c>
       <c r="D5" t="n">
         <v>95</v>
       </c>
       <c r="E5" t="n">
-        <v>95.29000000000001</v>
+        <v>95.95999999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>0.5206</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>COHESION</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Decision Tree</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Residual Bootstrap</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>95</v>
-      </c>
-      <c r="E6" t="n">
-        <v>95.45</v>
-      </c>
-      <c r="F6" t="n">
-        <v>6.797</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>MC</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Gradient Boosting</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Residual Bootstrap</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>95</v>
-      </c>
-      <c r="E7" t="n">
-        <v>95.29000000000001</v>
-      </c>
-      <c r="F7" t="n">
-        <v>12.845</v>
+        <v>12.9696</v>
       </c>
     </row>
   </sheetData>
@@ -2092,7 +1945,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2132,7 +1985,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.453110668964797</v>
+        <v>0.7959307651421913</v>
       </c>
     </row>
     <row r="3">
@@ -2146,11 +1999,11 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>depth_x_n60</t>
+          <t>soil_Sand-Other</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.1209340056766973</v>
+        <v>0.0794902494299472</v>
       </c>
     </row>
     <row r="4">
@@ -2164,11 +2017,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>depth_m</t>
+          <t>soil_Silty Sand(SM)</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.0808979262947378</v>
+        <v>0.0721855095079536</v>
       </c>
     </row>
     <row r="5">
@@ -2182,11 +2035,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>gwt_m</t>
+          <t>Nfield_sqrt</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.0580932223713152</v>
+        <v>0.0623432246388026</v>
       </c>
     </row>
     <row r="6">
@@ -2200,17 +2053,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>soil_Sand-Other</t>
+          <t>Nfield</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.0379359251006364</v>
+        <v>0.0603967838190859</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GAMMA_WET</t>
+          <t>SP_GR</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -2222,13 +2075,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.535936595019039</v>
+        <v>0.6742774463741588</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GAMMA_WET</t>
+          <t>SP_GR</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -2236,17 +2089,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>gwt_m</t>
+          <t>GWT(m)</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.3410203643313719</v>
+        <v>0.07880561234667049</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GAMMA_WET</t>
+          <t>SP_GR</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -2254,17 +2107,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>n60</t>
+          <t>Nfield_over_Depth(m)</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.0457403781456218</v>
+        <v>0.0291578604091859</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>GAMMA_WET</t>
+          <t>SP_GR</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -2272,17 +2125,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>depth_m</t>
+          <t>Depth(m)_x_Nfield</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.0272740829993686</v>
+        <v>0.0262115661292614</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GAMMA_WET</t>
+          <t>SP_GR</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -2290,17 +2143,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>n60_over_depth</t>
+          <t>Depth(m)</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.021032918666711</v>
+        <v>0.0233780275591464</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GAMMA_DRY</t>
+          <t>COHESION</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -2308,17 +2161,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>soil_Clay(CL)</t>
+          <t>soil_Silty Clay(CL)</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.5216262143629411</v>
+        <v>0.9425427891007528</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>GAMMA_DRY</t>
+          <t>COHESION</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -2326,17 +2179,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>gwt_m</t>
+          <t>Depth(m)</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.2404838614628265</v>
+        <v>0.1584866949061018</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>GAMMA_DRY</t>
+          <t>COHESION</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -2344,17 +2197,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>n60</t>
+          <t>GWT(m)</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.0364732581752716</v>
+        <v>0.0487541508645385</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GAMMA_DRY</t>
+          <t>COHESION</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -2362,17 +2215,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>soil_Silty Sand(SM)</t>
+          <t>Nfield_over_Depth(m)</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.0190637219693678</v>
+        <v>0.0231818975842873</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GAMMA_DRY</t>
+          <t>COHESION</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -2380,17 +2233,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>n60_over_depth</t>
+          <t>Depth(m)_x_Nfield</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.017888803811717</v>
+        <v>0.0050851461711039</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SP_GR</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2398,17 +2251,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>soil_Clay(CL)</t>
+          <t>GWT(m)</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.6687827325089707</v>
+        <v>0.18254824643196</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SP_GR</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -2416,17 +2269,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>layer_thickness_m</t>
+          <t>soil_Clay(CL)</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.07327123347978889</v>
+        <v>0.1346926821101606</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SP_GR</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -2434,17 +2287,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>depth_x_n60</t>
+          <t>Nfield_over_Depth(m)</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.0449544116941253</v>
+        <v>0.0848169943768088</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SP_GR</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -2452,17 +2305,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>soil_Sand(SM)</t>
+          <t>soil_Silty Clay(CL)</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.0439929440269882</v>
+        <v>0.0518002278344147</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SP_GR</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -2470,191 +2323,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>gwt_m</t>
+          <t>Depth(m)_x_Nfield</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.0291652571573149</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>COHESION</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>1</v>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>soil_Silty Clay(CL)</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>1.272256157226643</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>COHESION</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>2</v>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>depth_m</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>0.6565114899418771</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>COHESION</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>3</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>gwt_m</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>0.4433242181200666</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>COHESION</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>4</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>n60_over_depth</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>0.0725610791110675</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>COHESION</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>5</v>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>n60_log</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>0.0229382992736659</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>MC</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>1</v>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>gwt_m</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>0.6740424238097401</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>MC</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>2</v>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>soil_Clay(CL)</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>0.3191401937034929</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>MC</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>3</v>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>depth_x_n60</t>
-        </is>
-      </c>
-      <c r="D29" t="n">
-        <v>0.1558904196514836</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>MC</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>4</v>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>depth_m</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>0.08135013708955401</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>MC</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>5</v>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>soil_Silty Clay(CL)</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>0.0305361680798452</v>
+        <v>0.0430736042216539</v>
       </c>
     </row>
   </sheetData>
@@ -2668,7 +2341,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2706,133 +2379,87 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Gradient Boosting</t>
+          <t>Extra Trees</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.9455</v>
+        <v>0.9645</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0188</v>
+        <v>0.09229999999999999</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>No (p &lt; 0.05)</t>
+          <t>Approximately Normal</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GAMMA_WET</t>
+          <t>SP_GR</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.9399</v>
+        <v>0.9486</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0007</v>
+        <v>0.0008</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>No (p &lt; 0.05)</t>
+          <t>Non-normal (p &lt; 0.05)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GAMMA_DRY</t>
+          <t>COHESION</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>Extra Trees</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.9006999999999999</v>
+        <v>0.4893</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>No (p &lt; 0.05)</t>
+          <t>Non-normal (p &lt; 0.05)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SP_GR</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Extra Trees</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.8329</v>
+        <v>0.8879</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>No (p &lt; 0.05)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>COHESION</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Decision Tree</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>0.6776</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>No (p &lt; 0.05)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>MC</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Gradient Boosting</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>0.8582</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>No (p &lt; 0.05)</t>
+          <t>Non-normal (p &lt; 0.05)</t>
         </is>
       </c>
     </row>
@@ -2847,7 +2474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2885,7 +2512,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Gradient Boosting</t>
+          <t>Extra Trees</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2895,7 +2522,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Gradient Boosting</t>
+          <t>Extra Trees</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -2907,133 +2534,79 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GAMMA_WET</t>
+          <t>SP_GR</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>gamma_wet_best_model.pkl</t>
+          <t>sp_gr_best_model.pkl</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>gamma_wet_best_model.pkl</t>
+          <t>sp_gr_best_model.pkl</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GAMMA_DRY</t>
+          <t>COHESION</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>Extra Trees</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>gamma_dry_best_model.pkl</t>
+          <t>cohesion_best_model.pkl</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>Extra Trees</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>gamma_dry_best_model.pkl</t>
+          <t>cohesion_best_model.pkl</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SP_GR</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Extra Trees</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>sp_gr_best_model.pkl</t>
+          <t>mc_best_model.pkl</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Extra Trees</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
-        <is>
-          <t>sp_gr_best_model.pkl</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>COHESION</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Decision Tree</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>cohesion_best_model.pkl</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Gradient Boosting</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>cohesion_tool_model.pkl</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>MC</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Gradient Boosting</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>mc_best_model.pkl</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Gradient Boosting</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
         <is>
           <t>mc_best_model.pkl</t>
         </is>

</xml_diff>